<commit_message>
modified models and data
</commit_message>
<xml_diff>
--- a/semiconductor-ml/Data/All_Materials.xlsx
+++ b/semiconductor-ml/Data/All_Materials.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f8f36234d981261/Desktop/Research SemiConductor/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f8f36234d981261/Desktop/Research SemiConductor/Semiconductor-Research-Lab/semiconductor-ml/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="257" documentId="11_5D713EA59446360F62355476585DCE3A87470C4D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16590D42-99B2-4CE9-89E6-439D03FAF47B}"/>
+  <xr:revisionPtr revIDLastSave="258" documentId="11_5D713EA59446360F62355476585DCE3A87470C4D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BF5A88F-AA16-424C-9427-FCE10667EA06}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="All_Materials_Cleaned" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -165,7 +164,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="591">
   <si>
     <t>Material</t>
   </si>
@@ -1944,7 +1943,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1963,18 +1962,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -2024,7 +2011,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2038,9 +2025,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5113,7 +5097,7 @@
         <v>476</v>
       </c>
       <c r="Q14" s="3"/>
-      <c r="R14" s="7" t="s">
+      <c r="R14" s="5" t="s">
         <v>586</v>
       </c>
       <c r="S14" s="3" t="s">
@@ -5127,8 +5111,8 @@
       <c r="A15" t="s">
         <v>489</v>
       </c>
-      <c r="B15" t="s">
-        <v>504</v>
+      <c r="B15">
+        <v>2.56</v>
       </c>
       <c r="C15" t="s">
         <v>504</v>

</xml_diff>